<commit_message>
Ajustes código da reescala e testes
Ajustes na fitness e população inicial da reescala. Testes de reescala reiniciados. Criação de gráfico da quantidade de alterações por indivíduos nas gerações
</commit_message>
<xml_diff>
--- a/Testes/reescala/Teste populacao e gerações/Teste1/0_população_inicial.xlsx
+++ b/Testes/reescala/Teste populacao e gerações/Teste1/0_população_inicial.xlsx
@@ -2259,8 +2259,8 @@
       <c r="P15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q15" s="5" t="n">
-        <v>0</v>
+      <c r="Q15" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R15" s="4" t="n">
         <v>1</v>
@@ -4559,8 +4559,8 @@
       <c r="P35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q35" s="4" t="n">
-        <v>1</v>
+      <c r="Q35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R35" s="4" t="n">
         <v>1</v>
@@ -4568,23 +4568,23 @@
       <c r="S35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W35" s="5" t="n">
-        <v>0</v>
+      <c r="T35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="X35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y35" s="5" t="n">
-        <v>0</v>
+      <c r="Y35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Z35" s="5" t="n">
         <v>0</v>
@@ -4601,8 +4601,8 @@
       <c r="AD35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE35" s="5" t="n">
-        <v>0</v>
+      <c r="AE35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AF35" s="5" t="n">
         <v>0</v>
@@ -9667,8 +9667,8 @@
       <c r="T24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U24" s="5" t="n">
-        <v>0</v>
+      <c r="U24" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V24" s="5" t="n">
         <v>0</v>
@@ -11610,8 +11610,8 @@
       <c r="P41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q41" s="5" t="n">
-        <v>0</v>
+      <c r="Q41" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R41" s="5" t="n">
         <v>0</v>
@@ -12530,8 +12530,8 @@
       <c r="P49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Q49" s="4" t="n">
-        <v>1</v>
+      <c r="Q49" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R49" s="4" t="n">
         <v>1</v>
@@ -12539,35 +12539,35 @@
       <c r="S49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V49" s="5" t="n">
-        <v>0</v>
+      <c r="T49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V49" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="W49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X49" s="5" t="n">
-        <v>0</v>
+      <c r="X49" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Y49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC49" s="5" t="n">
-        <v>0</v>
+      <c r="Z49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD49" s="5" t="n">
         <v>0</v>
@@ -12575,14 +12575,14 @@
       <c r="AE49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH49" s="5" t="n">
-        <v>0</v>
+      <c r="AF49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH49" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AI49" s="5" t="n">
         <v>0</v>
@@ -14878,50 +14878,50 @@
       <c r="T14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="U14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W14" s="5" t="n">
-        <v>0</v>
+      <c r="U14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="X14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA14" s="5" t="n">
-        <v>0</v>
+      <c r="Y14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AB14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC14" s="5" t="n">
-        <v>0</v>
+      <c r="AC14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG14" s="5" t="n">
-        <v>0</v>
+      <c r="AE14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AH14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AI14" s="5" t="n">
-        <v>0</v>
+      <c r="AI14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ14" s="6">
         <f>SUM(F14:AI14)</f>
@@ -17511,8 +17511,8 @@
       <c r="P37" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q37" s="4" t="n">
-        <v>1</v>
+      <c r="Q37" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R37" s="4" t="n">
         <v>1</v>
@@ -17856,8 +17856,8 @@
       <c r="P40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Q40" s="5" t="n">
-        <v>0</v>
+      <c r="Q40" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R40" s="4" t="n">
         <v>1</v>
@@ -23615,8 +23615,8 @@
       <c r="G35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="4" t="n">
-        <v>1</v>
+      <c r="H35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I35" s="5" t="n">
         <v>0</v>
@@ -23645,11 +23645,11 @@
       <c r="Q35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" s="4" t="n">
-        <v>1</v>
+      <c r="R35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T35" s="5" t="n">
         <v>0</v>
@@ -23660,26 +23660,26 @@
       <c r="V35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W35" s="5" t="n">
-        <v>0</v>
+      <c r="W35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="X35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y35" s="5" t="n">
-        <v>0</v>
+      <c r="Y35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Z35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA35" s="5" t="n">
-        <v>0</v>
+      <c r="AA35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AB35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC35" s="5" t="n">
-        <v>0</v>
+      <c r="AC35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD35" s="5" t="n">
         <v>0</v>
@@ -23690,14 +23690,14 @@
       <c r="AF35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI35" s="5" t="n">
-        <v>0</v>
+      <c r="AG35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ35" s="6">
         <f>SUM(F35:AI35)</f>
@@ -28968,62 +28968,62 @@
       <c r="P26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" s="5" t="n">
-        <v>0</v>
+      <c r="Q26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="U26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="V26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB26" s="5" t="n">
-        <v>0</v>
+      <c r="V26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AC26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG26" s="5" t="n">
-        <v>0</v>
+      <c r="AD26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AH26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AI26" s="5" t="n">
-        <v>0</v>
+      <c r="AI26" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ26" s="6">
         <f>SUM(F26:AI26)</f>
@@ -30693,8 +30693,8 @@
       <c r="P41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q41" s="5" t="n">
-        <v>0</v>
+      <c r="Q41" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R41" s="5" t="n">
         <v>0</v>
@@ -33029,8 +33029,8 @@
       <c r="P6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" s="5" t="n">
-        <v>0</v>
+      <c r="Q6" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>1</v>
@@ -33961,8 +33961,8 @@
       <c r="T14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="U14" s="5" t="n">
-        <v>0</v>
+      <c r="U14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V14" s="5" t="n">
         <v>0</v>
@@ -33973,38 +33973,38 @@
       <c r="X14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="5" t="n">
-        <v>0</v>
+      <c r="Y14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Z14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA14" s="5" t="n">
-        <v>0</v>
+      <c r="AA14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AB14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC14" s="5" t="n">
-        <v>0</v>
+      <c r="AC14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI14" s="5" t="n">
-        <v>0</v>
+      <c r="AE14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ14" s="6">
         <f>SUM(F14:AI14)</f>
@@ -37514,8 +37514,8 @@
       <c r="P45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q45" s="4" t="n">
-        <v>1</v>
+      <c r="Q45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R45" s="4" t="n">
         <v>1</v>
@@ -40655,8 +40655,8 @@
       <c r="P17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q17" s="4" t="n">
-        <v>1</v>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R17" s="4" t="n">
         <v>1</v>
@@ -40670,14 +40670,14 @@
       <c r="U17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="V17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X17" s="5" t="n">
-        <v>0</v>
+      <c r="V17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Y17" s="5" t="n">
         <v>0</v>
@@ -40688,8 +40688,8 @@
       <c r="AA17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB17" s="5" t="n">
-        <v>0</v>
+      <c r="AB17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AC17" s="5" t="n">
         <v>0</v>
@@ -40697,20 +40697,20 @@
       <c r="AD17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE17" s="5" t="n">
-        <v>0</v>
+      <c r="AE17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AF17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG17" s="5" t="n">
-        <v>0</v>
+      <c r="AG17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AH17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AI17" s="5" t="n">
-        <v>0</v>
+      <c r="AI17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ17" s="6">
         <f>SUM(F17:AI17)</f>
@@ -43875,8 +43875,8 @@
       <c r="P45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q45" s="5" t="n">
-        <v>0</v>
+      <c r="Q45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R45" s="4" t="n">
         <v>1</v>
@@ -48511,8 +48511,8 @@
       <c r="P30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q30" s="5" t="n">
-        <v>0</v>
+      <c r="Q30" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R30" s="4" t="n">
         <v>1</v>
@@ -48680,8 +48680,8 @@
       <c r="AH31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AI31" s="5" t="n">
-        <v>0</v>
+      <c r="AI31" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AJ31" s="6">
         <f>SUM(F31:AI31)</f>
@@ -50236,8 +50236,8 @@
       <c r="P45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q45" s="4" t="n">
-        <v>1</v>
+      <c r="Q45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R45" s="4" t="n">
         <v>1</v>
@@ -50245,53 +50245,53 @@
       <c r="S45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U45" s="5" t="n">
-        <v>0</v>
+      <c r="T45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W45" s="5" t="n">
-        <v>0</v>
+      <c r="W45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="X45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z45" s="5" t="n">
-        <v>0</v>
+      <c r="Y45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AA45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB45" s="5" t="n">
-        <v>0</v>
+      <c r="AB45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AC45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI45" s="4" t="n">
-        <v>1</v>
+      <c r="AD45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AJ45" s="6">
         <f>SUM(F45:AI45)</f>
@@ -53033,7 +53033,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" s="7" t="n">
         <v>0</v>
@@ -55217,53 +55217,53 @@
       <c r="P33" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" s="4" t="n">
-        <v>1</v>
+      <c r="Q33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X33" s="4" t="n">
-        <v>1</v>
+      <c r="U33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X33" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Y33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z33" s="5" t="n">
-        <v>0</v>
+      <c r="Z33" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AA33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB33" s="5" t="n">
-        <v>0</v>
+      <c r="AB33" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AC33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD33" s="5" t="n">
-        <v>0</v>
+      <c r="AD33" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AE33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF33" s="5" t="n">
-        <v>0</v>
+      <c r="AF33" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AG33" s="5" t="n">
         <v>0</v>
@@ -58473,8 +58473,8 @@
       <c r="P6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" s="5" t="n">
-        <v>0</v>
+      <c r="Q6" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>1</v>
@@ -62586,8 +62586,8 @@
       <c r="G42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="5" t="n">
-        <v>0</v>
+      <c r="H42" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="I42" s="5" t="n">
         <v>0</v>
@@ -62613,8 +62613,8 @@
       <c r="P42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q42" s="4" t="n">
-        <v>1</v>
+      <c r="Q42" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R42" s="4" t="n">
         <v>1</v>

</xml_diff>